<commit_message>
fix(lineup): fix QNED 85/86 duplicate pairs and 100/115-inch size misclassification across European retailers
</commit_message>
<xml_diff>
--- a/data/price tracker_EU_2026 0912_v1.xlsx
+++ b/data/price tracker_EU_2026 0912_v1.xlsx
@@ -50900,7 +50900,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>55</v>
+        <v>115</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -50978,7 +50978,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -51017,7 +51017,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>115</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -51329,7 +51329,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -53860,7 +53860,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -53899,7 +53899,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -53938,7 +53938,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>55</v>
+        <v>115</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>

</xml_diff>